<commit_message>
Novo registro: cleiton.teste | MRVH - PARQUE DOS PRINCIPES - BA/SA | 19/10/2026 16:34:50
</commit_message>
<xml_diff>
--- a/inventario_equipamentos.xlsx
+++ b/inventario_equipamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,24 +493,64 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>54354545646546546546</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>78787878787878</t>
-        </is>
+      <c r="G2" t="n">
+        <v>5.435454564654654e+19</v>
+      </c>
+      <c r="H2" t="n">
+        <v>78787878787878</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Celular obra 360°</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>13131313131313</t>
+      <c r="J2" t="n">
+        <v>13131313131313</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>19/10/2026 16:34:50</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cleiton.teste</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MRVH - PARQUE DOS PRINCIPES - BA/SA</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>54354545646546546546cs\fdjskabdjflalsfkas</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>78787878787878asdgfasdgfnasdlknflks</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>13131313131313sadgga</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Novo registro: pollyanna.bento@mrv.com.br | E148 - URB PARQUE DAS CORES - SP/CP | 19/10/2026 16:38:44
</commit_message>
<xml_diff>
--- a/inventario_equipamentos.xlsx
+++ b/inventario_equipamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,11 @@
           <t>Celular_1_Patrimônio</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Desktop_2_Patrimônio</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -507,6 +512,7 @@
       <c r="J2" t="n">
         <v>13131313131313</v>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -551,6 +557,58 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>13131313131313sadgga</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19/10/2026 16:38:44</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pollyanna.bento@mrv.com.br</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>E148 - URB PARQUE DAS CORES - SP/CP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>9FDADSFF</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>6DG666HG</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>666X6VV</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1SFGGF66</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Novo registro: cleiton.souza | Q005 - CASTELLO DI VENETO - MS/CG | 19/10/2026 16:44:44
</commit_message>
<xml_diff>
--- a/inventario_equipamentos.xlsx
+++ b/inventario_equipamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:Z5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,81 @@
           <t>Desktop_2_Patrimônio</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Desktop_3_Patrimônio</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Desktop_4_Patrimônio</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Desktop_5_Patrimônio</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Notebook_2_Patrimônio</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Notebook_3_Patrimônio</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Celular_2_Tipo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Celular_2_Patrimônio</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Celular_3_Tipo</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Celular_3_Patrimônio</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Celular_4_Tipo</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Celular_4_Patrimônio</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Celular_5_Tipo</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Celular_5_Patrimônio</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Celular_6_Tipo</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Celular_6_Patrimônio</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -513,6 +588,21 @@
         <v>13131313131313</v>
       </c>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,6 +650,21 @@
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -609,6 +714,147 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>1SFGGF66</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>19/10/2026 16:44:44</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cleiton.souza</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Q005 - CASTELLO DI VENETO - MS/CG</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>tgsreg</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>qDASGDFGHBJ</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>AD\ZFSDGXFHCGVHB</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>sfdgsfdhbfshg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>qwerty</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>asdfghjklç</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>zxcvbnm,asdfghjklçqweqwertyuio</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>qdafsgdfhghbj</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SDASFGDHFJJ</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>|xaZSDXBCFNVH</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>\AZVXDBCFNVGB</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>|azSDXCFVGBN</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Qwartfgyhujikl</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>awszdxfcgvbhjnmklpiuyhtfdres</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Novo registro: cleiton.teste | CASASMAIS SANTA IRIA - SP/RP | 19/10/2026 17:01:57
</commit_message>
<xml_diff>
--- a/inventario_equipamentos.xlsx
+++ b/inventario_equipamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z5"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -858,6 +858,92 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>19/10/2026 17:01:57</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cleiton.teste</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CASASMAIS SANTA IRIA - SP/RP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>13131313131313sadgga</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>QWSETDRYFTUGYHU</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>EWARSETDRYFTUGYH</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Wqeawrsetdry</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>wqaezxedgtcrfh</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>waersetdryft</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Novo registro: teste.teste@gmail.com.br | E148 - RESIDENCIAL CORES DA ILHA - SP/CP | 19/10/2026 17:46:37
</commit_message>
<xml_diff>
--- a/inventario_equipamentos.xlsx
+++ b/inventario_equipamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -989,6 +989,77 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>19/10/2026 17:46:37</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>E148 - RESIDENCIAL CORES DA ILHA - SP/CP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>112555</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>323255</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>355966</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Celular obra 360°</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>123569</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>teste.teste@gmail.com.br</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Novo registro: pollyanna.bento@mrv.com.br | Q018 - SENSIA HORIZON - PR/CR | 19/10/2026 20:04:01
</commit_message>
<xml_diff>
--- a/inventario_equipamentos.xlsx
+++ b/inventario_equipamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1060,6 +1060,77 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>19/10/2026 20:04:01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Q018 - SENSIA HORIZON - PR/CR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>123569</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>123569</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Celular padrão</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>125698</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>563951</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>pollyanna.bento@mrv.com.br</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>